<commit_message>
fixed data being saved, as well as updated readme
</commit_message>
<xml_diff>
--- a/prediction_score.xlsx
+++ b/prediction_score.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Score Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPY" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AAPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSFT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AMZN" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="META" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +474,1558 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-02-24 00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>696.77</v>
+      </c>
+      <c r="C2" t="n">
+        <v>704.12</v>
+      </c>
+      <c r="D2" t="n">
+        <v>688.64</v>
+      </c>
+      <c r="E2" t="n">
+        <v>685.48</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02-25 00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>684.87</v>
+      </c>
+      <c r="C3" t="n">
+        <v>693.01</v>
+      </c>
+      <c r="D3" t="n">
+        <v>677.52</v>
+      </c>
+      <c r="E3" t="n">
+        <v>691.26</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-02-28 00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>683.48</v>
+      </c>
+      <c r="C4" t="n">
+        <v>692.96</v>
+      </c>
+      <c r="D4" t="n">
+        <v>674.91</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-27 00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>651.26</v>
+      </c>
+      <c r="C5" t="n">
+        <v>662.15</v>
+      </c>
+      <c r="D5" t="n">
+        <v>639.22</v>
+      </c>
+      <c r="E5" t="n">
+        <v>634.09</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-28 00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>667.71</v>
+      </c>
+      <c r="C6" t="n">
+        <v>680.23</v>
+      </c>
+      <c r="D6" t="n">
+        <v>656.39</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:42</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>646.0700000000001</v>
+      </c>
+      <c r="C7" t="n">
+        <v>665.29</v>
+      </c>
+      <c r="D7" t="n">
+        <v>631.86</v>
+      </c>
+      <c r="E7" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-08 23:29</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>663.51</v>
+      </c>
+      <c r="C8" t="n">
+        <v>680.97</v>
+      </c>
+      <c r="D8" t="n">
+        <v>650.61</v>
+      </c>
+      <c r="E8" t="n">
+        <v>676.01</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-13 00:26</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>649.66</v>
+      </c>
+      <c r="C9" t="n">
+        <v>663.38</v>
+      </c>
+      <c r="D9" t="n">
+        <v>639.52</v>
+      </c>
+      <c r="E9" t="n">
+        <v>686.1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-14 02:44</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>655.38</v>
+      </c>
+      <c r="C10" t="n">
+        <v>668.72</v>
+      </c>
+      <c r="D10" t="n">
+        <v>645.51</v>
+      </c>
+      <c r="E10" t="n">
+        <v>694.46</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-16 21:24</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>672.78</v>
+      </c>
+      <c r="C11" t="n">
+        <v>684.53</v>
+      </c>
+      <c r="D11" t="n">
+        <v>664.09</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Prediction Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Predicted Close</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Close</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Error %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>In Range</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Direction Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-02-24 00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>265.8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>277.86</v>
+      </c>
+      <c r="D2" t="n">
+        <v>254.89</v>
+      </c>
+      <c r="E2" t="n">
+        <v>272.14</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02-25 00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>276.95</v>
+      </c>
+      <c r="C3" t="n">
+        <v>288.96</v>
+      </c>
+      <c r="D3" t="n">
+        <v>268.08</v>
+      </c>
+      <c r="E3" t="n">
+        <v>274.23</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-02-28 00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>266.13</v>
+      </c>
+      <c r="C4" t="n">
+        <v>273.19</v>
+      </c>
+      <c r="D4" t="n">
+        <v>260.91</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-27 00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>257.49</v>
+      </c>
+      <c r="C5" t="n">
+        <v>261.73</v>
+      </c>
+      <c r="D5" t="n">
+        <v>253.65</v>
+      </c>
+      <c r="E5" t="n">
+        <v>248.8</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-28 00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>259.38</v>
+      </c>
+      <c r="C6" t="n">
+        <v>263.3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>255.83</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:42</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>262.64</v>
+      </c>
+      <c r="C7" t="n">
+        <v>270.04</v>
+      </c>
+      <c r="D7" t="n">
+        <v>257.17</v>
+      </c>
+      <c r="E7" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-08 23:30</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>269.21</v>
+      </c>
+      <c r="C8" t="n">
+        <v>277.49</v>
+      </c>
+      <c r="D8" t="n">
+        <v>263.09</v>
+      </c>
+      <c r="E8" t="n">
+        <v>258.9</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-13 00:25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>268.65</v>
+      </c>
+      <c r="C9" t="n">
+        <v>276.71</v>
+      </c>
+      <c r="D9" t="n">
+        <v>262.69</v>
+      </c>
+      <c r="E9" t="n">
+        <v>259.2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-14 02:44</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>267.8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>276.02</v>
+      </c>
+      <c r="D10" t="n">
+        <v>261.73</v>
+      </c>
+      <c r="E10" t="n">
+        <v>258.83</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-16 21:24</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>268.04</v>
+      </c>
+      <c r="C11" t="n">
+        <v>275.24</v>
+      </c>
+      <c r="D11" t="n">
+        <v>262.71</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Prediction Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Predicted Close</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Close</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Error %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>In Range</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Direction Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-02-24 00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>386.59</v>
+      </c>
+      <c r="C2" t="n">
+        <v>392.93</v>
+      </c>
+      <c r="D2" t="n">
+        <v>380.86</v>
+      </c>
+      <c r="E2" t="n">
+        <v>389</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02-25 00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>393.28</v>
+      </c>
+      <c r="C3" t="n">
+        <v>400.17</v>
+      </c>
+      <c r="D3" t="n">
+        <v>385.67</v>
+      </c>
+      <c r="E3" t="n">
+        <v>400.6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-02-28 00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>382.7</v>
+      </c>
+      <c r="C4" t="n">
+        <v>396.18</v>
+      </c>
+      <c r="D4" t="n">
+        <v>370.51</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-27 00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>388.94</v>
+      </c>
+      <c r="C5" t="n">
+        <v>396.7</v>
+      </c>
+      <c r="D5" t="n">
+        <v>381.92</v>
+      </c>
+      <c r="E5" t="n">
+        <v>356.77</v>
+      </c>
+      <c r="F5" t="n">
+        <v>9.02</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-28 00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>393.46</v>
+      </c>
+      <c r="C6" t="n">
+        <v>401.15</v>
+      </c>
+      <c r="D6" t="n">
+        <v>386.5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:42</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>337.75</v>
+      </c>
+      <c r="C7" t="n">
+        <v>349.41</v>
+      </c>
+      <c r="D7" t="n">
+        <v>329.13</v>
+      </c>
+      <c r="E7" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-08 23:29</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>398.27</v>
+      </c>
+      <c r="C8" t="n">
+        <v>410.03</v>
+      </c>
+      <c r="D8" t="n">
+        <v>389.58</v>
+      </c>
+      <c r="E8" t="n">
+        <v>374.33</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-13 00:26</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>376.61</v>
+      </c>
+      <c r="C9" t="n">
+        <v>382.93</v>
+      </c>
+      <c r="D9" t="n">
+        <v>371.94</v>
+      </c>
+      <c r="E9" t="n">
+        <v>384.37</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-14 02:44</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>361.76</v>
+      </c>
+      <c r="C10" t="n">
+        <v>367.97</v>
+      </c>
+      <c r="D10" t="n">
+        <v>357.17</v>
+      </c>
+      <c r="E10" t="n">
+        <v>393.11</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-16 21:23</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>446.44</v>
+      </c>
+      <c r="C11" t="n">
+        <v>583.58</v>
+      </c>
+      <c r="D11" t="n">
+        <v>324.84</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Prediction Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Predicted Close</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Close</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Error %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>In Range</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Direction Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-28 00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>215.82</v>
+      </c>
+      <c r="C2" t="n">
+        <v>222.93</v>
+      </c>
+      <c r="D2" t="n">
+        <v>207.96</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:42</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>234.55</v>
+      </c>
+      <c r="C3" t="n">
+        <v>245.81</v>
+      </c>
+      <c r="D3" t="n">
+        <v>226.23</v>
+      </c>
+      <c r="E3" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-08 23:29</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>224.42</v>
+      </c>
+      <c r="C4" t="n">
+        <v>232.99</v>
+      </c>
+      <c r="D4" t="n">
+        <v>218.08</v>
+      </c>
+      <c r="E4" t="n">
+        <v>221.25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-13 00:26</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>211.33</v>
+      </c>
+      <c r="C5" t="n">
+        <v>218.43</v>
+      </c>
+      <c r="D5" t="n">
+        <v>206.09</v>
+      </c>
+      <c r="E5" t="n">
+        <v>239.89</v>
+      </c>
+      <c r="F5" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-14 02:44</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>225.39</v>
+      </c>
+      <c r="C6" t="n">
+        <v>233.64</v>
+      </c>
+      <c r="D6" t="n">
+        <v>219.29</v>
+      </c>
+      <c r="E6" t="n">
+        <v>249.02</v>
+      </c>
+      <c r="F6" t="n">
+        <v>9.49</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-16 21:23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>231.42</v>
+      </c>
+      <c r="C7" t="n">
+        <v>314.75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>167.54</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Prediction Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Predicted Close</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Close</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Error %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>In Range</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Direction Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-08 23:29</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>618</v>
+      </c>
+      <c r="C2" t="n">
+        <v>658.1900000000001</v>
+      </c>
+      <c r="D2" t="n">
+        <v>588.29</v>
+      </c>
+      <c r="E2" t="n">
+        <v>612.42</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-13 00:26</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>693.48</v>
+      </c>
+      <c r="C3" t="n">
+        <v>732.25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>664.83</v>
+      </c>
+      <c r="E3" t="n">
+        <v>634.53</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9.289999999999999</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-14 02:44</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>734.16</v>
+      </c>
+      <c r="C4" t="n">
+        <v>774.47</v>
+      </c>
+      <c r="D4" t="n">
+        <v>704.36</v>
+      </c>
+      <c r="E4" t="n">
+        <v>662.49</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10.82</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-16 21:24</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>672.92</v>
+      </c>
+      <c r="C5" t="n">
+        <v>705.39</v>
+      </c>
+      <c r="D5" t="n">
+        <v>648.92</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
created a build, as well as added editing of model
The application is now a .exe file
</commit_message>
<xml_diff>
--- a/prediction_score.xlsx
+++ b/prediction_score.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -786,10 +786,10 @@
         <v>639.58</v>
       </c>
       <c r="E11" t="n">
-        <v>700.71</v>
+        <v>701.66</v>
       </c>
       <c r="F11" t="n">
-        <v>3.98</v>
+        <v>4.11</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -805,34 +805,66 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-17 03:13</t>
+          <t>2026-04-17 03:14</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>681.75</v>
+        <v>681.8</v>
       </c>
       <c r="C12" t="n">
-        <v>733.74</v>
+        <v>733.79</v>
       </c>
       <c r="D12" t="n">
-        <v>655.61</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>655.65</v>
+      </c>
+      <c r="E12" t="n">
+        <v>710.14</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3.99</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-18 18:12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>671.04</v>
+      </c>
+      <c r="C13" t="n">
+        <v>679.8099999999999</v>
+      </c>
+      <c r="D13" t="n">
+        <v>664.5599999999999</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -849,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1206,10 +1238,10 @@
         <v>249.65</v>
       </c>
       <c r="E11" t="n">
-        <v>264.18</v>
+        <v>263.4</v>
       </c>
       <c r="F11" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1225,34 +1257,66 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-17 03:13</t>
+          <t>2026-04-17 03:14</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>269.12</v>
+        <v>269.14</v>
       </c>
       <c r="C12" t="n">
-        <v>274.1</v>
+        <v>274.11</v>
       </c>
       <c r="D12" t="n">
-        <v>254.51</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>254.52</v>
+      </c>
+      <c r="E12" t="n">
+        <v>270.23</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.4</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-18 18:12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>265.61</v>
+      </c>
+      <c r="C13" t="n">
+        <v>273.07</v>
+      </c>
+      <c r="D13" t="n">
+        <v>260.1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1269,7 +1333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1626,10 +1690,10 @@
         <v>343.25</v>
       </c>
       <c r="E11" t="n">
-        <v>417.79</v>
+        <v>420.26</v>
       </c>
       <c r="F11" t="n">
-        <v>6.86</v>
+        <v>6.24</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1645,34 +1709,66 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-17 03:13</t>
+          <t>2026-04-17 03:14</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>479.2</v>
+        <v>479.17</v>
       </c>
       <c r="C12" t="n">
-        <v>599.09</v>
+        <v>599.05</v>
       </c>
       <c r="D12" t="n">
-        <v>370.73</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>370.7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>422.79</v>
+      </c>
+      <c r="F12" t="n">
+        <v>13.33</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-18 18:12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>484.91</v>
+      </c>
+      <c r="C13" t="n">
+        <v>502.14</v>
+      </c>
+      <c r="D13" t="n">
+        <v>472.17</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1689,7 +1785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1914,10 +2010,10 @@
         <v>224.38</v>
       </c>
       <c r="E7" t="n">
-        <v>248.26</v>
+        <v>249.7</v>
       </c>
       <c r="F7" t="n">
-        <v>6.79</v>
+        <v>7.33</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1926,41 +2022,73 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-17 03:13</t>
+          <t>2026-04-17 03:14</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>234.67</v>
+        <v>234.74</v>
       </c>
       <c r="C8" t="n">
-        <v>306.21</v>
+        <v>306.31</v>
       </c>
       <c r="D8" t="n">
-        <v>178.2</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>178.26</v>
+      </c>
+      <c r="E8" t="n">
+        <v>250.56</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.31</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-18 18:12</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>233.47</v>
+      </c>
+      <c r="C9" t="n">
+        <v>241.96</v>
+      </c>
+      <c r="D9" t="n">
+        <v>227.19</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1977,7 +2105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2134,10 +2262,10 @@
         <v>649.04</v>
       </c>
       <c r="E5" t="n">
-        <v>673.39</v>
+        <v>676.87</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05</v>
+        <v>0.57</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2165,22 +2293,54 @@
       <c r="D6" t="n">
         <v>624.46</v>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E6" t="n">
+        <v>688.55</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6.29</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-18 18:12</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>708.71</v>
+      </c>
+      <c r="C7" t="n">
+        <v>735.87</v>
+      </c>
+      <c r="D7" t="n">
+        <v>688.63</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
loading screen on start up
</commit_message>
<xml_diff>
--- a/prediction_score.xlsx
+++ b/prediction_score.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -841,34 +841,66 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-20 22:03</t>
+          <t>2026-04-20 22:04</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>665.85</v>
+        <v>665.92</v>
       </c>
       <c r="C13" t="n">
-        <v>673.41</v>
+        <v>729.4299999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>660.26</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>627.65</v>
+      </c>
+      <c r="E13" t="n">
+        <v>708.72</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6.04</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:13</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>682.37</v>
+      </c>
+      <c r="C14" t="n">
+        <v>692.08</v>
+      </c>
+      <c r="D14" t="n">
+        <v>675.1900000000001</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -885,7 +917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1329,34 +1361,66 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-20 22:03</t>
+          <t>2026-04-20 22:04</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>270.09</v>
+        <v>270.13</v>
       </c>
       <c r="C14" t="n">
-        <v>277.89</v>
+        <v>276.36</v>
       </c>
       <c r="D14" t="n">
-        <v>264.33</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>256.39</v>
+      </c>
+      <c r="E14" t="n">
+        <v>273.05</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.07</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:13</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>270.78</v>
+      </c>
+      <c r="C15" t="n">
+        <v>281.53</v>
+      </c>
+      <c r="D15" t="n">
+        <v>262.82</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1373,7 +1437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1817,34 +1881,66 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-20 22:03</t>
+          <t>2026-04-20 22:04</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>441.53</v>
+        <v>441.55</v>
       </c>
       <c r="C14" t="n">
-        <v>457.43</v>
+        <v>457.47</v>
       </c>
       <c r="D14" t="n">
-        <v>429.77</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>429.79</v>
+      </c>
+      <c r="E14" t="n">
+        <v>418.07</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5.62</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:13</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>482.63</v>
+      </c>
+      <c r="C15" t="n">
+        <v>502.16</v>
+      </c>
+      <c r="D15" t="n">
+        <v>468.19</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1861,7 +1957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2173,34 +2269,66 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-20 22:03</t>
+          <t>2026-04-20 22:04</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>226.58</v>
+        <v>226.48</v>
       </c>
       <c r="C10" t="n">
-        <v>233.92</v>
+        <v>277.91</v>
       </c>
       <c r="D10" t="n">
-        <v>219.94</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>190.6</v>
+      </c>
+      <c r="E10" t="n">
+        <v>248.28</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8.779999999999999</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:13</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>226.68</v>
+      </c>
+      <c r="C11" t="n">
+        <v>232.25</v>
+      </c>
+      <c r="D11" t="n">
+        <v>222.57</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2217,7 +2345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2461,34 +2589,66 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-20 22:03</t>
+          <t>2026-04-20 22:04</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>669.9400000000001</v>
+        <v>669.92</v>
       </c>
       <c r="C8" t="n">
-        <v>694.62</v>
+        <v>738.05</v>
       </c>
       <c r="D8" t="n">
-        <v>651.7</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>568.29</v>
+      </c>
+      <c r="E8" t="n">
+        <v>670.91</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.15</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:13</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>736.47</v>
+      </c>
+      <c r="C9" t="n">
+        <v>764.1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>716.04</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
bug fix for errornous data
</commit_message>
<xml_diff>
--- a/prediction_score.xlsx
+++ b/prediction_score.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSFT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AMZN" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="META" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVDA" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -805,17 +806,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-18 18:17</t>
+          <t>2026-04-18 21:33</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>659.35</v>
+        <v>658.85</v>
       </c>
       <c r="C12" t="n">
-        <v>667.96</v>
+        <v>667.46</v>
       </c>
       <c r="D12" t="n">
-        <v>652.98</v>
+        <v>652.49</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -841,102 +842,264 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-20 22:04</t>
+          <t>2026-04-19 23:40</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>665.92</v>
+        <v>658.64</v>
       </c>
       <c r="C13" t="n">
-        <v>729.4299999999999</v>
+        <v>667.24</v>
       </c>
       <c r="D13" t="n">
-        <v>627.65</v>
-      </c>
-      <c r="E13" t="n">
-        <v>708.72</v>
-      </c>
-      <c r="F13" t="n">
-        <v>6.04</v>
+        <v>652.28</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-25 19:13</t>
+          <t>2026-04-20 21:44</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>682.29</v>
+        <v>664.2</v>
       </c>
       <c r="C14" t="n">
-        <v>741.63</v>
+        <v>671.76</v>
       </c>
       <c r="D14" t="n">
-        <v>651.48</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Not Available</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>658.61</v>
+      </c>
+      <c r="E14" t="n">
+        <v>708.72</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6.28</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-27 20:11</t>
+          <t>2026-04-22 22:53</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>680.77</v>
+        <v>682.54</v>
       </c>
       <c r="C15" t="n">
-        <v>690.46</v>
+        <v>757.55</v>
       </c>
       <c r="D15" t="n">
-        <v>673.61</v>
-      </c>
-      <c r="E15" t="inlineStr">
+        <v>636.46</v>
+      </c>
+      <c r="E15" t="n">
+        <v>711.21</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-23 18:39</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>679.95</v>
+      </c>
+      <c r="C16" t="n">
+        <v>687.92</v>
+      </c>
+      <c r="D16" t="n">
+        <v>674.0599999999999</v>
+      </c>
+      <c r="E16" t="n">
+        <v>708.45</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-24 15:45</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>676.64</v>
+      </c>
+      <c r="C17" t="n">
+        <v>743.61</v>
+      </c>
+      <c r="D17" t="n">
+        <v>638.64</v>
+      </c>
+      <c r="E17" t="n">
+        <v>713.9400000000001</v>
+      </c>
+      <c r="F17" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:19</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>677.23</v>
+      </c>
+      <c r="C18" t="n">
+        <v>686.86</v>
+      </c>
+      <c r="D18" t="n">
+        <v>670.11</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:45</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>676.77</v>
+      </c>
+      <c r="C19" t="n">
+        <v>736.13</v>
+      </c>
+      <c r="D19" t="n">
+        <v>647.9299999999999</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-27 20:20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -953,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1169,23 +1332,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-07 20:42</t>
+          <t>2026-04-07 00:00</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>262.64</v>
+        <v>262.33</v>
       </c>
       <c r="C7" t="n">
-        <v>270.04</v>
+        <v>269.71</v>
       </c>
       <c r="D7" t="n">
-        <v>257.17</v>
+        <v>256.87</v>
       </c>
       <c r="E7" t="n">
         <v>253.5</v>
       </c>
       <c r="F7" t="n">
-        <v>3.61</v>
+        <v>3.48</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1201,27 +1364,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-08 23:30</t>
+          <t>2026-04-08 00:00</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>269.21</v>
+        <v>257.4</v>
       </c>
       <c r="C8" t="n">
-        <v>277.49</v>
+        <v>265.59</v>
       </c>
       <c r="D8" t="n">
-        <v>263.09</v>
+        <v>251.35</v>
       </c>
       <c r="E8" t="n">
         <v>258.9</v>
       </c>
       <c r="F8" t="n">
-        <v>3.98</v>
+        <v>0.58</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1233,23 +1396,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-13 00:25</t>
+          <t>2026-04-14 00:00</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>268.65</v>
+        <v>267.59</v>
       </c>
       <c r="C9" t="n">
-        <v>276.71</v>
+        <v>275.8</v>
       </c>
       <c r="D9" t="n">
-        <v>262.69</v>
+        <v>261.52</v>
       </c>
       <c r="E9" t="n">
-        <v>259.2</v>
+        <v>258.83</v>
       </c>
       <c r="F9" t="n">
-        <v>3.65</v>
+        <v>3.38</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1265,27 +1428,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-14 02:44</t>
+          <t>2026-04-16 00:00</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>267.8</v>
+        <v>268.1</v>
       </c>
       <c r="C10" t="n">
-        <v>276.02</v>
+        <v>275.3</v>
       </c>
       <c r="D10" t="n">
-        <v>261.73</v>
+        <v>262.77</v>
       </c>
       <c r="E10" t="n">
-        <v>258.83</v>
+        <v>263.4</v>
       </c>
       <c r="F10" t="n">
-        <v>3.47</v>
+        <v>1.78</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1297,23 +1460,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-16 21:26</t>
+          <t>2026-04-17 00:00</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>268.14</v>
+        <v>269.14</v>
       </c>
       <c r="C11" t="n">
-        <v>277.85</v>
+        <v>274.11</v>
       </c>
       <c r="D11" t="n">
-        <v>249.65</v>
+        <v>254.52</v>
       </c>
       <c r="E11" t="n">
-        <v>263.4</v>
+        <v>270.23</v>
       </c>
       <c r="F11" t="n">
-        <v>1.8</v>
+        <v>0.4</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1322,102 +1485,102 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-17 03:14</t>
+          <t>2026-04-18 00:00</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>269.14</v>
+        <v>265.62</v>
       </c>
       <c r="C12" t="n">
-        <v>274.11</v>
+        <v>273.08</v>
       </c>
       <c r="D12" t="n">
-        <v>254.52</v>
-      </c>
-      <c r="E12" t="n">
-        <v>270.23</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.4</v>
+        <v>260.11</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-18 18:17</t>
+          <t>2026-04-20 00:00</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>265.7</v>
+        <v>266.35</v>
       </c>
       <c r="C13" t="n">
-        <v>273.16</v>
+        <v>273.82</v>
       </c>
       <c r="D13" t="n">
-        <v>260.19</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Not Available</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>260.82</v>
+      </c>
+      <c r="E13" t="n">
+        <v>273.05</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.45</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-20 22:04</t>
+          <t>2026-04-22 00:00</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>270.13</v>
+        <v>265.74</v>
       </c>
       <c r="C14" t="n">
-        <v>276.36</v>
+        <v>272.26</v>
       </c>
       <c r="D14" t="n">
-        <v>256.39</v>
+        <v>253.11</v>
       </c>
       <c r="E14" t="n">
-        <v>273.05</v>
+        <v>273.17</v>
       </c>
       <c r="F14" t="n">
-        <v>1.07</v>
+        <v>2.72</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1429,70 +1592,164 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-25 19:13</t>
+          <t>2026-04-23 18:39</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>270.94</v>
+        <v>271.46</v>
       </c>
       <c r="C15" t="n">
-        <v>277.44</v>
+        <v>281.61</v>
       </c>
       <c r="D15" t="n">
-        <v>258.1</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Not Available</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>263.96</v>
+      </c>
+      <c r="E15" t="n">
+        <v>273.43</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.72</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-27 20:10</t>
+          <t>2026-04-24 15:45</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>270.92</v>
+        <v>274.88</v>
       </c>
       <c r="C16" t="n">
-        <v>281.68</v>
+        <v>283.24</v>
       </c>
       <c r="D16" t="n">
-        <v>262.96</v>
-      </c>
-      <c r="E16" t="inlineStr">
+        <v>264.19</v>
+      </c>
+      <c r="E16" t="n">
+        <v>271.06</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:19</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>267.35</v>
+      </c>
+      <c r="C17" t="n">
+        <v>277.97</v>
+      </c>
+      <c r="D17" t="n">
+        <v>259.49</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:45</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>267.34</v>
+      </c>
+      <c r="C18" t="n">
+        <v>275.01</v>
+      </c>
+      <c r="D18" t="n">
+        <v>257.39</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-27 20:20</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1509,7 +1766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1725,23 +1982,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-07 20:42</t>
+          <t>2026-04-07 00:00</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>337.75</v>
+        <v>338.36</v>
       </c>
       <c r="C7" t="n">
-        <v>349.41</v>
+        <v>350.04</v>
       </c>
       <c r="D7" t="n">
-        <v>329.13</v>
+        <v>329.73</v>
       </c>
       <c r="E7" t="n">
         <v>372.29</v>
       </c>
       <c r="F7" t="n">
-        <v>9.279999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1757,27 +2014,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-08 23:29</t>
+          <t>2026-04-08 00:00</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>398.27</v>
+        <v>380.96</v>
       </c>
       <c r="C8" t="n">
-        <v>410.03</v>
+        <v>394.18</v>
       </c>
       <c r="D8" t="n">
-        <v>389.58</v>
+        <v>371.19</v>
       </c>
       <c r="E8" t="n">
         <v>374.33</v>
       </c>
       <c r="F8" t="n">
-        <v>6.4</v>
+        <v>1.77</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1789,23 +2046,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-13 00:26</t>
+          <t>2026-04-14 00:00</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>376.61</v>
+        <v>362.99</v>
       </c>
       <c r="C9" t="n">
-        <v>382.93</v>
+        <v>369.26</v>
       </c>
       <c r="D9" t="n">
-        <v>371.94</v>
+        <v>358.36</v>
       </c>
       <c r="E9" t="n">
-        <v>384.37</v>
+        <v>393.11</v>
       </c>
       <c r="F9" t="n">
-        <v>2.02</v>
+        <v>7.66</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1814,62 +2071,62 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-14 02:44</t>
+          <t>2026-04-16 00:00</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>361.76</v>
+        <v>445.54</v>
       </c>
       <c r="C10" t="n">
-        <v>367.97</v>
+        <v>582.39</v>
       </c>
       <c r="D10" t="n">
-        <v>357.17</v>
+        <v>324.18</v>
       </c>
       <c r="E10" t="n">
-        <v>393.11</v>
+        <v>420.26</v>
       </c>
       <c r="F10" t="n">
-        <v>7.97</v>
+        <v>6.02</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-16 21:26</t>
+          <t>2026-04-17 00:00</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>446.47</v>
+        <v>479.17</v>
       </c>
       <c r="C11" t="n">
-        <v>560.3</v>
+        <v>599.05</v>
       </c>
       <c r="D11" t="n">
-        <v>343.25</v>
+        <v>370.7</v>
       </c>
       <c r="E11" t="n">
-        <v>420.26</v>
+        <v>422.79</v>
       </c>
       <c r="F11" t="n">
-        <v>6.24</v>
+        <v>13.34</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1885,117 +2142,117 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-17 03:14</t>
+          <t>2026-04-18 00:00</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>479.17</v>
+        <v>485.15</v>
       </c>
       <c r="C12" t="n">
-        <v>599.05</v>
+        <v>502.4</v>
       </c>
       <c r="D12" t="n">
-        <v>370.7</v>
-      </c>
-      <c r="E12" t="n">
-        <v>422.79</v>
-      </c>
-      <c r="F12" t="n">
-        <v>13.33</v>
+        <v>472.41</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-18 18:17</t>
+          <t>2026-04-20 00:00</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>485.14</v>
+        <v>487</v>
       </c>
       <c r="C13" t="n">
-        <v>502.39</v>
+        <v>504.31</v>
       </c>
       <c r="D13" t="n">
-        <v>472.4</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Not Available</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>474.2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>418.07</v>
+      </c>
+      <c r="F13" t="n">
+        <v>16.49</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-20 22:04</t>
+          <t>2026-04-22 00:00</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>441.55</v>
+        <v>480.84</v>
       </c>
       <c r="C14" t="n">
-        <v>457.47</v>
+        <v>586.16</v>
       </c>
       <c r="D14" t="n">
-        <v>429.79</v>
+        <v>376.48</v>
       </c>
       <c r="E14" t="n">
-        <v>418.07</v>
+        <v>432.92</v>
       </c>
       <c r="F14" t="n">
-        <v>5.62</v>
+        <v>11.07</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-25 19:13</t>
+          <t>2026-04-25 19:19</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>482.59</v>
+        <v>418.07</v>
       </c>
       <c r="C15" t="n">
-        <v>502.12</v>
+        <v>434.99</v>
       </c>
       <c r="D15" t="n">
-        <v>468.15</v>
+        <v>405.56</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2021,34 +2278,70 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-27 20:10</t>
+          <t>2026-04-26 18:45</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>482.15</v>
+        <v>418.35</v>
       </c>
       <c r="C16" t="n">
-        <v>501.66</v>
+        <v>475.2</v>
       </c>
       <c r="D16" t="n">
-        <v>467.72</v>
+        <v>346.71</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-27 20:19</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>418.11</v>
+      </c>
+      <c r="C17" t="n">
+        <v>435.03</v>
+      </c>
+      <c r="D17" t="n">
+        <v>405.6</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2065,7 +2358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2341,17 +2634,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-18 18:17</t>
+          <t>2026-04-18 21:33</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>233.39</v>
+        <v>233.38</v>
       </c>
       <c r="C9" t="n">
-        <v>241.88</v>
+        <v>241.87</v>
       </c>
       <c r="D9" t="n">
-        <v>227.12</v>
+        <v>227.11</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2377,102 +2670,270 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-20 22:04</t>
+          <t>2026-04-19 23:40</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>226.48</v>
+        <v>233.25</v>
       </c>
       <c r="C10" t="n">
-        <v>277.91</v>
+        <v>241.74</v>
       </c>
       <c r="D10" t="n">
-        <v>190.6</v>
-      </c>
-      <c r="E10" t="n">
-        <v>248.28</v>
-      </c>
-      <c r="F10" t="n">
-        <v>8.779999999999999</v>
+        <v>226.98</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-25 19:13</t>
+          <t>2026-04-20 21:43</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>226.87</v>
+        <v>227.05</v>
       </c>
       <c r="C11" t="n">
-        <v>232.44</v>
+        <v>234.4</v>
       </c>
       <c r="D11" t="n">
-        <v>222.75</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Not Available</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>220.39</v>
+      </c>
+      <c r="E11" t="n">
+        <v>248.28</v>
+      </c>
+      <c r="F11" t="n">
+        <v>8.550000000000001</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-27 20:11</t>
+          <t>2026-04-22 22:53</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>224.12</v>
+        <v>246.38</v>
       </c>
       <c r="C12" t="n">
-        <v>229.62</v>
+        <v>307.41</v>
       </c>
       <c r="D12" t="n">
-        <v>220.05</v>
-      </c>
-      <c r="E12" t="inlineStr">
+        <v>203.36</v>
+      </c>
+      <c r="E12" t="n">
+        <v>255.36</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-23 18:39</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>242.52</v>
+      </c>
+      <c r="C13" t="n">
+        <v>248.73</v>
+      </c>
+      <c r="D13" t="n">
+        <v>237.92</v>
+      </c>
+      <c r="E13" t="n">
+        <v>255.08</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-24 15:45</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>239.82</v>
+      </c>
+      <c r="C14" t="n">
+        <v>287.38</v>
+      </c>
+      <c r="D14" t="n">
+        <v>211.89</v>
+      </c>
+      <c r="E14" t="n">
+        <v>263.99</v>
+      </c>
+      <c r="F14" t="n">
+        <v>9.16</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:19</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>224.04</v>
+      </c>
+      <c r="C15" t="n">
+        <v>229.55</v>
+      </c>
+      <c r="D15" t="n">
+        <v>219.97</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:45</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>222.29</v>
+      </c>
+      <c r="C16" t="n">
+        <v>258.85</v>
+      </c>
+      <c r="D16" t="n">
+        <v>204.9</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-27 20:19</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>225.75</v>
+      </c>
+      <c r="C17" t="n">
+        <v>231.29</v>
+      </c>
+      <c r="D17" t="n">
+        <v>221.65</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2489,7 +2950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2697,17 +3158,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-18 18:17</t>
+          <t>2026-04-18 21:33</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>708.92</v>
+        <v>708.72</v>
       </c>
       <c r="C7" t="n">
-        <v>736.09</v>
+        <v>735.88</v>
       </c>
       <c r="D7" t="n">
-        <v>688.84</v>
+        <v>688.65</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2733,102 +3194,398 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-20 22:04</t>
+          <t>2026-04-19 23:40</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>669.92</v>
+        <v>709.8200000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>738.05</v>
+        <v>737.02</v>
       </c>
       <c r="D8" t="n">
-        <v>568.29</v>
-      </c>
-      <c r="E8" t="n">
-        <v>670.91</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.15</v>
+        <v>689.71</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-25 19:13</t>
+          <t>2026-04-20 21:44</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>736.46</v>
+        <v>669.42</v>
       </c>
       <c r="C9" t="n">
-        <v>764.09</v>
+        <v>694.02</v>
       </c>
       <c r="D9" t="n">
-        <v>716.03</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Not Available</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>651.23</v>
+      </c>
+      <c r="E9" t="n">
+        <v>670.91</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.22</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-27 20:11</t>
+          <t>2026-04-22 22:53</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>738.6900000000001</v>
+        <v>655</v>
       </c>
       <c r="C10" t="n">
-        <v>766.41</v>
+        <v>699.78</v>
       </c>
       <c r="D10" t="n">
-        <v>718.2</v>
-      </c>
-      <c r="E10" t="inlineStr">
+        <v>574.27</v>
+      </c>
+      <c r="E10" t="n">
+        <v>674.72</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-23 18:39</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>657.55</v>
+      </c>
+      <c r="C11" t="n">
+        <v>678.1799999999999</v>
+      </c>
+      <c r="D11" t="n">
+        <v>638.87</v>
+      </c>
+      <c r="E11" t="n">
+        <v>659.15</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-24 15:45</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>713.36</v>
+      </c>
+      <c r="C12" t="n">
+        <v>752.04</v>
+      </c>
+      <c r="D12" t="n">
+        <v>640.74</v>
+      </c>
+      <c r="E12" t="n">
+        <v>675.03</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-25 19:19</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>742.78</v>
+      </c>
+      <c r="C13" t="n">
+        <v>770.65</v>
+      </c>
+      <c r="D13" t="n">
+        <v>722.1799999999999</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:45</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>743.38</v>
+      </c>
+      <c r="C14" t="n">
+        <v>777.08</v>
+      </c>
+      <c r="D14" t="n">
+        <v>672.5</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>471.02</v>
+      </c>
+      <c r="C15" t="n">
+        <v>492.37</v>
+      </c>
+      <c r="D15" t="n">
+        <v>426.11</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Prediction Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Predicted Close</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Close</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Error %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>In Range</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Direction Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-26 18:46</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>195.64</v>
+      </c>
+      <c r="C2" t="n">
+        <v>201.23</v>
+      </c>
+      <c r="D2" t="n">
+        <v>191.51</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-27 20:15</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>195.45</v>
+      </c>
+      <c r="C3" t="n">
+        <v>201.03</v>
+      </c>
+      <c r="D3" t="n">
+        <v>191.32</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
cleaned up repeated functions, as well as redundant variables
</commit_message>
<xml_diff>
--- a/prediction_score.xlsx
+++ b/prediction_score.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1078,28 +1078,66 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-27 20:20</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
+          <t>2026-04-27 00:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="C20" t="n">
+        <v>20.46</v>
+      </c>
+      <c r="D20" t="n">
+        <v>18.01</v>
+      </c>
+      <c r="E20" t="n">
+        <v>715.17</v>
+      </c>
+      <c r="F20" t="n">
+        <v>97.37</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-01 12:53</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>697.99</v>
+      </c>
+      <c r="C21" t="n">
+        <v>706.5599999999999</v>
+      </c>
+      <c r="D21" t="n">
+        <v>691.66</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1116,7 +1154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1728,28 +1766,66 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-27 20:20</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
+          <t>2026-04-27 00:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>136.16</v>
+      </c>
+      <c r="C19" t="n">
+        <v>140.07</v>
+      </c>
+      <c r="D19" t="n">
+        <v>131.09</v>
+      </c>
+      <c r="E19" t="n">
+        <v>267.61</v>
+      </c>
+      <c r="F19" t="n">
+        <v>49.12</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-01 12:53</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>265.68</v>
+      </c>
+      <c r="C20" t="n">
+        <v>273.12</v>
+      </c>
+      <c r="D20" t="n">
+        <v>260.19</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1766,7 +1842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2314,34 +2390,66 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-27 20:19</t>
+          <t>2026-04-27 20:21</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>418.11</v>
+        <v>417.97</v>
       </c>
       <c r="C17" t="n">
-        <v>435.03</v>
+        <v>474.77</v>
       </c>
       <c r="D17" t="n">
-        <v>405.6</v>
-      </c>
-      <c r="E17" t="inlineStr">
+        <v>346.4</v>
+      </c>
+      <c r="E17" t="n">
+        <v>424.82</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-01 12:54</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>428.41</v>
+      </c>
+      <c r="C18" t="n">
+        <v>446.78</v>
+      </c>
+      <c r="D18" t="n">
+        <v>411.79</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2358,7 +2466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2906,34 +3014,66 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-27 20:19</t>
+          <t>2026-04-27 20:21</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>225.75</v>
+        <v>225.96</v>
       </c>
       <c r="C17" t="n">
-        <v>231.29</v>
+        <v>263.13</v>
       </c>
       <c r="D17" t="n">
-        <v>221.65</v>
-      </c>
-      <c r="E17" t="inlineStr">
+        <v>208.29</v>
+      </c>
+      <c r="E17" t="n">
+        <v>261.12</v>
+      </c>
+      <c r="F17" t="n">
+        <v>13.47</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-01 12:53</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>236.22</v>
+      </c>
+      <c r="C18" t="n">
+        <v>244.46</v>
+      </c>
+      <c r="D18" t="n">
+        <v>230.14</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2950,7 +3090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3442,22 +3582,54 @@
       <c r="D15" t="n">
         <v>426.11</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" t="n">
+        <v>678.62</v>
+      </c>
+      <c r="F15" t="n">
+        <v>30.59</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-01 12:53</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>672.0599999999999</v>
+      </c>
+      <c r="C16" t="n">
+        <v>696.58</v>
+      </c>
+      <c r="D16" t="n">
+        <v>644.95</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3474,7 +3646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3558,34 +3730,66 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-27 20:15</t>
+          <t>2026-04-27 20:21</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>195.45</v>
+        <v>195.41</v>
       </c>
       <c r="C3" t="n">
-        <v>201.03</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>191.32</v>
-      </c>
-      <c r="E3" t="inlineStr">
+        <v>191.29</v>
+      </c>
+      <c r="E3" t="n">
+        <v>216.61</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-01 12:53</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>198.05</v>
+      </c>
+      <c r="C4" t="n">
+        <v>208.32</v>
+      </c>
+      <c r="D4" t="n">
+        <v>188.76</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
redo of the data parsing as it was inconsistent, leading to wrong predictions occasionally
</commit_message>
<xml_diff>
--- a/prediction_score.xlsx
+++ b/prediction_score.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1110,34 +1110,138 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-01 12:53</t>
+          <t>2026-05-02 00:00</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>697.99</v>
+        <v>701.96</v>
       </c>
       <c r="C21" t="n">
-        <v>706.5599999999999</v>
+        <v>773.4</v>
       </c>
       <c r="D21" t="n">
-        <v>691.66</v>
+        <v>668.66</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-03 23:59</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>704.49</v>
+      </c>
+      <c r="C22" t="n">
+        <v>776.1900000000001</v>
+      </c>
+      <c r="D22" t="n">
+        <v>671.0700000000001</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-04 20:40</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>703.09</v>
+      </c>
+      <c r="C23" t="n">
+        <v>711.1799999999999</v>
+      </c>
+      <c r="D23" t="n">
+        <v>697.1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>718.01</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-05 12:56</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>703.58</v>
+      </c>
+      <c r="C24" t="n">
+        <v>777.36</v>
+      </c>
+      <c r="D24" t="n">
+        <v>669.25</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1154,7 +1258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1798,34 +1902,138 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-01 12:53</t>
+          <t>2026-05-02 00:00</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>265.68</v>
+        <v>271.49</v>
       </c>
       <c r="C20" t="n">
-        <v>273.12</v>
+        <v>280.73</v>
       </c>
       <c r="D20" t="n">
-        <v>260.19</v>
+        <v>260.59</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-03 23:59</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>269.95</v>
+      </c>
+      <c r="C21" t="n">
+        <v>279.14</v>
+      </c>
+      <c r="D21" t="n">
+        <v>259.11</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-04 20:40</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>269.67</v>
+      </c>
+      <c r="C22" t="n">
+        <v>276.96</v>
+      </c>
+      <c r="D22" t="n">
+        <v>264.28</v>
+      </c>
+      <c r="E22" t="n">
+        <v>276.83</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-05 12:56</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>265.99</v>
+      </c>
+      <c r="C23" t="n">
+        <v>274.67</v>
+      </c>
+      <c r="D23" t="n">
+        <v>255.76</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1842,7 +2050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2422,34 +2630,138 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-01 12:54</t>
+          <t>2026-05-02 00:00</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>428.41</v>
+        <v>388.2</v>
       </c>
       <c r="C18" t="n">
-        <v>446.78</v>
+        <v>435.01</v>
       </c>
       <c r="D18" t="n">
-        <v>411.79</v>
+        <v>327.92</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-03 23:59</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>395.71</v>
+      </c>
+      <c r="C19" t="n">
+        <v>443.43</v>
+      </c>
+      <c r="D19" t="n">
+        <v>334.26</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-04 20:40</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>416.94</v>
+      </c>
+      <c r="C20" t="n">
+        <v>434.19</v>
+      </c>
+      <c r="D20" t="n">
+        <v>401.34</v>
+      </c>
+      <c r="E20" t="n">
+        <v>413.62</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-05 12:56</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>450.51</v>
+      </c>
+      <c r="C21" t="n">
+        <v>497.38</v>
+      </c>
+      <c r="D21" t="n">
+        <v>385.93</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2466,7 +2778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3046,34 +3358,138 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-01 12:53</t>
+          <t>2026-05-02 00:00</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>236.22</v>
+        <v>218.25</v>
       </c>
       <c r="C18" t="n">
-        <v>244.46</v>
+        <v>258.33</v>
       </c>
       <c r="D18" t="n">
-        <v>230.14</v>
+        <v>204.58</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-03 23:59</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>215.08</v>
+      </c>
+      <c r="C19" t="n">
+        <v>254.58</v>
+      </c>
+      <c r="D19" t="n">
+        <v>201.61</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-04 20:40</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>213.19</v>
+      </c>
+      <c r="C20" t="n">
+        <v>220.06</v>
+      </c>
+      <c r="D20" t="n">
+        <v>208.11</v>
+      </c>
+      <c r="E20" t="n">
+        <v>272.05</v>
+      </c>
+      <c r="F20" t="n">
+        <v>21.64</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-05 12:56</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>230.16</v>
+      </c>
+      <c r="C21" t="n">
+        <v>280.48</v>
+      </c>
+      <c r="D21" t="n">
+        <v>213.1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3090,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3602,34 +4018,138 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-01 12:53</t>
+          <t>2026-05-02 00:00</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>672.0599999999999</v>
+        <v>665.08</v>
       </c>
       <c r="C16" t="n">
-        <v>696.58</v>
+        <v>750.46</v>
       </c>
       <c r="D16" t="n">
-        <v>644.95</v>
+        <v>591.84</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-03 23:59</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>660.3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>745.0700000000001</v>
+      </c>
+      <c r="D17" t="n">
+        <v>587.59</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-04 20:40</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>659.13</v>
+      </c>
+      <c r="C18" t="n">
+        <v>686.49</v>
+      </c>
+      <c r="D18" t="n">
+        <v>628.88</v>
+      </c>
+      <c r="E18" t="n">
+        <v>610.41</v>
+      </c>
+      <c r="F18" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-05 12:56</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>662.6900000000001</v>
+      </c>
+      <c r="C19" t="n">
+        <v>726.11</v>
+      </c>
+      <c r="D19" t="n">
+        <v>587.45</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3646,7 +4166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3762,34 +4282,138 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-01 12:53</t>
+          <t>2026-05-02 00:00</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>198.05</v>
+        <v>198.33</v>
       </c>
       <c r="C4" t="n">
-        <v>208.32</v>
+        <v>208.15</v>
       </c>
       <c r="D4" t="n">
-        <v>188.76</v>
+        <v>187.47</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-03 23:59</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>198.68</v>
+      </c>
+      <c r="C5" t="n">
+        <v>208.51</v>
+      </c>
+      <c r="D5" t="n">
+        <v>187.8</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-04 20:40</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>198.9</v>
+      </c>
+      <c r="C6" t="n">
+        <v>208.74</v>
+      </c>
+      <c r="D6" t="n">
+        <v>188.01</v>
+      </c>
+      <c r="E6" t="n">
+        <v>198.48</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-05 12:56</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>203.07</v>
+      </c>
+      <c r="C7" t="n">
+        <v>212.54</v>
+      </c>
+      <c r="D7" t="n">
+        <v>192.61</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>